<commit_message>
Updated app.py with less comments and more summarized docstring.Evaluation file will be dealt with later in details
</commit_message>
<xml_diff>
--- a/docs/genie-evaluation/Avanti_Genie_evaluation.xlsx
+++ b/docs/genie-evaluation/Avanti_Genie_evaluation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0d44ed6bc9ff19ff/NFT - Internship/Avanti/Proposed Solution/Azure Databricks/avanti-command-centre/docs/genie-evaluation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_2590E4722B3D3E71C4409ABE8070AF38911AFF1D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{49CA3BCB-E1B4-1B4F-BC3B-C01EF2EE9E3B}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="11_2590E4722B3D3E71C4409ABE8070AF38911AFF1D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B064775C-4C9E-EB49-B297-75E04C1BED11}"/>
   <bookViews>
-    <workbookView xWindow="53400" yWindow="600" windowWidth="19200" windowHeight="21000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="53400" yWindow="600" windowWidth="19200" windowHeight="21000" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -951,7 +951,7 @@
       <c r="C13" s="8"/>
       <c r="D13" s="8"/>
     </row>
-    <row r="14" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" ht="56" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="10" t="s">
         <v>23</v>
       </c>
@@ -961,7 +961,7 @@
       <c r="C14" s="8"/>
       <c r="D14" s="8"/>
     </row>
-    <row r="15" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="10" t="s">
         <v>25</v>
       </c>

</xml_diff>

<commit_message>
Made changes in the references, documentations, screenshots to serve it as a project history on github
</commit_message>
<xml_diff>
--- a/docs/genie-evaluation/Avanti_Genie_evaluation.xlsx
+++ b/docs/genie-evaluation/Avanti_Genie_evaluation.xlsx
@@ -8,16 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0d44ed6bc9ff19ff/NFT - Internship/Avanti/Proposed Solution/Azure Databricks/avanti-command-centre/docs/genie-evaluation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="11_2590E4722B3D3E71C4409ABE8070AF38911AFF1D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B064775C-4C9E-EB49-B297-75E04C1BED11}"/>
+  <xr:revisionPtr revIDLastSave="48" documentId="11_2590E4722B3D3E71C4409ABE8070AF38911AFF1D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7591D3B2-98E4-734D-82ED-1CCFDD9A26D0}"/>
   <bookViews>
-    <workbookView xWindow="53400" yWindow="600" windowWidth="19200" windowHeight="21000" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34200" yWindow="600" windowWidth="38400" windowHeight="21000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
-    <sheet name="Baseline" sheetId="2" r:id="rId2"/>
-    <sheet name="After curation" sheetId="3" r:id="rId3"/>
-    <sheet name="Findings" sheetId="4" r:id="rId4"/>
-    <sheet name="Quality levers" sheetId="5" r:id="rId5"/>
+    <sheet name="After curation" sheetId="3" r:id="rId2"/>
+    <sheet name="Findings" sheetId="4" r:id="rId3"/>
+    <sheet name="Quality levers" sheetId="5" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -40,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="108">
   <si>
     <t>Genie evaluation — Avanti Command Centre</t>
   </si>
@@ -150,69 +149,21 @@
     <t>Percentage</t>
   </si>
   <si>
-    <t>DECISION</t>
-  </si>
-  <si>
-    <t>Genie is sufficient?</t>
-  </si>
-  <si>
-    <t>If yes: wrap the Conversations API, always show the SQL, keep this benchmark as a regression test. If no: build a tool-calling layer over the marts, with this benchmark as the acceptance criterion.</t>
-  </si>
-  <si>
-    <t>Reason 1</t>
-  </si>
-  <si>
-    <t>Reason 2</t>
-  </si>
-  <si>
-    <t>Reason 3</t>
-  </si>
-  <si>
     <t>CAVEAT — the data is synthetic. Clinics are assigned round-robin by the generator, so genuine outliers are unlikely and apparent differences are largely artefacts of interacting modulo cycles. Any business 'insight' here is a rendering test, not a finding. Five questions is enough to make a build-or-wrap decision; not enough to claim an accuracy figure.</t>
   </si>
   <si>
-    <t>Baseline — bare space, no instructions</t>
-  </si>
-  <si>
-    <t>Run before adding instructions or sample queries, to establish whether the mart design alone is self-explanatory. Yellow cells are to be completed.</t>
-  </si>
-  <si>
     <t>#</t>
   </si>
   <si>
     <t>Question (as asked)</t>
   </si>
   <si>
-    <t>Expected answer</t>
-  </si>
-  <si>
     <t>Score</t>
   </si>
   <si>
     <t>Generated SQL</t>
   </si>
   <si>
-    <t>Why it scored that</t>
-  </si>
-  <si>
-    <t>Which clinic is least profitable?</t>
-  </si>
-  <si>
-    <t>Which month was least profitable?</t>
-  </si>
-  <si>
-    <t>Which discipline generates the most revenue?</t>
-  </si>
-  <si>
-    <t>How much revenue have we lost to appointments not attended?</t>
-  </si>
-  <si>
-    <t>Show me revenue by clinic by month</t>
-  </si>
-  <si>
-    <t>If a clean baseline was not captured before instructions were added, say so here rather than reconstructing one. A missing baseline is more honest than an invented one.</t>
-  </si>
-  <si>
     <t>After curation — instructions and sample queries added</t>
   </si>
   <si>
@@ -249,15 +200,9 @@
     <t>Conversation context silently narrows scope</t>
   </si>
   <si>
-    <t>Asked 'give me the least profitable clinic'. Generated SQL contained WHERE month_start = '2026-08-01'. Nothing in the question mentioned August — the scope was inherited from an earlier turn. Correcting it produced WHERE month_start &lt;= '2026-08-01', still excluding two months.</t>
-  </si>
-  <si>
     <t>A manager asking three questions may have the third answered under constraints from the first, with no indication. For a client-facing tool that is a correctness problem, not a usability one.</t>
   </si>
   <si>
-    <t>Fresh conversation per question when evaluating. In the app, consider making continuation explicit rather than the default.</t>
-  </si>
-  <si>
     <t>Grain ambiguity produced a confidently wrong answer</t>
   </si>
   <si>
@@ -273,9 +218,6 @@
     <t>Correct figures, incorrect narrative</t>
   </si>
   <si>
-    <t>'Newtown's direct costs are disproportionately high relative to its revenue.' Costs were roughly flat across all six clinics (~190K); revenue varied twofold (290K to 641K). The cause was LOW REVENUE, not high costs.</t>
-  </si>
-  <si>
     <t>The strongest argument for the app rendering the table and the SQL rather than the summary alone. A reader who skims the prose takes away the wrong conclusion.</t>
   </si>
   <si>
@@ -321,9 +263,6 @@
     <t>Hardcoded dates in generated SQL</t>
   </si>
   <si>
-    <t>A refinement suggested WHERE month_start &lt; '2026-10-01'. It encodes today's data boundary as a literal, so it silently excludes November data the moment it lands. It was also redundant — appointments_completed &gt; 0 already excludes future months.</t>
-  </si>
-  <si>
     <t>The model observed that October rows were empty and encoded THAT SPECIFIC FACT rather than the rule behind it. Same class of error as a hardcoded catalog name in a config file.</t>
   </si>
   <si>
@@ -384,14 +323,135 @@
     <t>Least significant of the five.</t>
   </si>
   <si>
-    <t>METHOD NOTE — the first pass at this evaluation was not an evaluation. Instructions were changed, the failing question re-asked, improvement observed, and the change kept. That demonstrates one question got better; it says nothing about whether the change helped generally or broke something that previously worked. The correct loop: collect real questions, write ground-truth SQL agreed with the business, baseline, change ONE thing, re-measure, keep or revert. Genie Agents has a benchmarking feature that takes question-plus-expected-SQL pairs — that should have been step one.</t>
+    <t>Tell me the least profitable clinic in terms of margin</t>
+  </si>
+  <si>
+    <t>Tell me the least profitable month in terms of margin.</t>
+  </si>
+  <si>
+    <t>Give me the list of the least utilized practitioners.</t>
+  </si>
+  <si>
+    <t>What is the overall revenue lost because of DNA (appointments not attended)? Don't show clinic-wise or month-wise data.</t>
+  </si>
+  <si>
+    <t>SELECT
+  `clinic_name`,
+  `state`,
+  SUM(`revenue`) AS total_revenue,
+  SUM(`direct_cost`) AS total_direct_cost,
+  SUM(`margin`) AS total_margin,
+  ROUND(SUM(`margin`) / NULLIF(SUM(`revenue`), 0) * 100, 2) AS margin_pct,
+  SUM(`appointments_completed`) AS total_appointments_completed,
+  COUNT(DISTINCT `month_start`) AS months_active
+FROM
+  `avanti_dev`.`gold`.`mart_clinic_monthly`
+WHERE
+  `appointments_completed` &gt; 0
+GROUP BY
+  `clinic_name`,
+  `state`
+ORDER BY
+  margin_pct ASC</t>
+  </si>
+  <si>
+    <t>SELECT
+  `month_start`,
+  `month_label`,
+  SUM(`revenue`) AS total_revenue,
+  SUM(`direct_cost`) AS total_direct_cost,
+  SUM(`margin`) AS total_margin,
+  CASE
+    WHEN SUM(`revenue`) = 0 THEN NULL
+    ELSE ROUND(SUM(`margin`) / NULLIF(SUM(`revenue`), 0) * 100
+  END AS margin_pct,
+  SUM(`appointments_completed`) AS appointments_completed
+FROM
+  `avanti_dev`.`gold`.`mart_clinic_monthly`
+WHERE
+  `appointments_completed` &gt; 0
+GROUP BY
+  `month_start`,
+  `month_label`
+ORDER BY
+  `month_start` ASC</t>
+  </si>
+  <si>
+    <t>SELECT
+  `practitioner_name`,
+  `discipline`,
+  ROUND(AVG(`utilisation_pct`) * 100, 1) AS avg_utilisation_pct,
+  SUM(`delivered_hours`) AS total_delivered_hours,
+  SUM(`available_hours`) AS total_available_hours,
+  SUM(`appointments_completed`) AS total_appointments_completed,
+  ROUND(SUM(`revenue`), 0) AS total_revenue
+FROM
+  avanti_dev.gold.`mart_practitioner_monthly`
+WHERE
+  `practitioner_name` IS NOT NULL
+  AND `practitioner_name` NOT IN ('unknown', 'Unknown', 'N/A', 'Other')
+  AND `available_hours` &gt; 0
+GROUP BY
+  `practitioner_name`,
+  `discipline`
+ORDER BY
+  avg_utilisation_pct ASC
+LIMIT 20</t>
+  </si>
+  <si>
+    <t>SELECT
+  SUM(`revenue_lost_to_dna`) AS total_revenue_lost_to_dna,
+  SUM(`appointments_dna`) AS total_dna_appointments,
+  SUM(`appointments_total`) AS total_appointments,
+  ROUND(SUM(`appointments_dna`) / NULLIF(SUM(`appointments_total`), 0) * 100, 2) AS overall_dna_rate
+FROM
+  `avanti_dev`.`gold`.`mart_clinic_monthly`</t>
+  </si>
+  <si>
+    <t>The ground-truth query that was updated has no record since that was not copied first</t>
+  </si>
+  <si>
+    <t>No Change</t>
+  </si>
+  <si>
+    <t>Asked 'give me the least profitable clinic'. Generated SQL contained WHERE month_start = '2026-08-01'. Nothing in the question mentioned August — the scope was inherited from an earlier turn. Correcting it produced WHERE month_start &lt;= '2026-08-01', still excluding two months. This is about when Genie was used without any mention of schema or table.</t>
+  </si>
+  <si>
+    <t>I wouldn't call this a fix but fresh conversation per question when evaluating resolved this problem. This is related to General Genie Agent not the one in the application that I created.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Newtown's direct costs are disproportionately high relative to its revenue.' Costs were roughly flat across all six clinics (~190K); revenue varied twofold (290K to 641K). The cause was </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FF444444"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>LOW REVENUE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF444444"/>
+        <rFont val="Arial"/>
+        <charset val="1"/>
+      </rPr>
+      <t>, not high costs.</t>
+    </r>
+  </si>
+  <si>
+    <t>A refinement suggested WHERE month_start &lt; '2026-10-01'. It encoded  today's data boundary as a literal, so it silently excludes November data the moment it lands. It was also redundant — appointments_completed &gt; 0 already excludes future months.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -440,7 +500,20 @@
     <font>
       <sz val="9"/>
       <name val="Courier New"/>
-      <charset val="1"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF444444"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF444444"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -511,18 +584,6 @@
   </cellStyleXfs>
   <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -547,24 +608,36 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -650,6 +723,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -831,7 +908,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -840,261 +917,212 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
     </row>
     <row r="2" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="6"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
     </row>
     <row r="5" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="8"/>
-      <c r="D5" s="9" t="s">
+      <c r="C5" s="4"/>
+      <c r="D5" s="5" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="8"/>
-      <c r="D6" s="9" t="s">
+      <c r="C6" s="4"/>
+      <c r="D6" s="5" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="8"/>
-      <c r="D7" s="9"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="5"/>
     </row>
     <row r="8" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="8"/>
-      <c r="D8" s="9" t="s">
+      <c r="C8" s="4"/>
+      <c r="D8" s="5" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="8"/>
-      <c r="D9" s="9" t="s">
+      <c r="C9" s="4"/>
+      <c r="D9" s="5" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="8"/>
-      <c r="D10" s="9" t="s">
+      <c r="C10" s="4"/>
+      <c r="D10" s="5" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
     </row>
     <row r="13" spans="1:4" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="10" t="s">
+      <c r="A13" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
     </row>
     <row r="14" spans="1:4" ht="56" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="10" t="s">
+      <c r="A14" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C14" s="8"/>
-      <c r="D14" s="8"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
     </row>
     <row r="15" spans="1:4" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="10" t="s">
+      <c r="A15" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="5" t="s">
+      <c r="A17" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B17" s="6"/>
-      <c r="C17" s="6"/>
-      <c r="D17" s="6"/>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
     </row>
     <row r="18" spans="1:4" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="11"/>
-      <c r="B18" s="11" t="s">
+      <c r="A18" s="7"/>
+      <c r="B18" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C18" s="11" t="s">
+      <c r="C18" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="D18" s="11" t="s">
+      <c r="D18" s="7" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="7" t="s">
+      <c r="A19" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="12">
-        <f>SUM(Baseline!D6:D10)</f>
-        <v>0</v>
-      </c>
-      <c r="C19" s="12">
-        <f>SUM('After curation'!E6:E10)</f>
-        <v>0</v>
-      </c>
-      <c r="D19" s="8" t="s">
+      <c r="B19" s="8">
+        <v>5</v>
+      </c>
+      <c r="C19" s="8">
+        <v>8</v>
+      </c>
+      <c r="D19" s="4" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="7" t="s">
+      <c r="A20" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B20" s="12">
-        <f>COUNT(Baseline!D6:D10)*2</f>
-        <v>0</v>
-      </c>
-      <c r="C20" s="12">
-        <f>COUNT('After curation'!E6:E10)*2</f>
-        <v>0</v>
-      </c>
-      <c r="D20" s="8" t="s">
+      <c r="B20" s="8">
+        <v>8</v>
+      </c>
+      <c r="C20" s="8">
+        <v>8</v>
+      </c>
+      <c r="D20" s="4" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="7" t="s">
+      <c r="A21" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B21" s="13" t="str">
+      <c r="B21" s="9">
         <f>IFERROR(B19/B20,"")</f>
-        <v/>
-      </c>
-      <c r="C21" s="13" t="str">
+        <v>0.625</v>
+      </c>
+      <c r="C21" s="9">
         <f>IFERROR(C19/C20,"")</f>
-        <v/>
-      </c>
-      <c r="D21" s="8"/>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D21" s="4"/>
+    </row>
+    <row r="24" spans="1:4" ht="45.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="B23" s="6"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
-    </row>
-    <row r="24" spans="1:4" ht="45.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="B24" s="14"/>
-      <c r="C24" s="8"/>
-      <c r="D24" s="9" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-    </row>
-    <row r="26" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-    </row>
-    <row r="27" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
-    </row>
-    <row r="29" spans="1:4" ht="45.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B29" s="1"/>
-      <c r="C29" s="1"/>
-      <c r="D29" s="1"/>
+      <c r="B24" s="16"/>
+      <c r="C24" s="16"/>
+      <c r="D24" s="16"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A29:D29"/>
+  <mergeCells count="3">
+    <mergeCell ref="A24:D24"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="B25:D25"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="B27:D27"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -1102,142 +1130,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="4" width="8" customWidth="1"/>
-    <col min="5" max="5" width="52" customWidth="1"/>
-    <col min="6" max="6" width="46" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-    </row>
-    <row r="2" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-    </row>
-    <row r="5" spans="1:6" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="B5" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="D5" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="E5" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="F5" s="11" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="54" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="12">
-        <v>1</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="C6" s="14"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="17"/>
-    </row>
-    <row r="7" spans="1:6" ht="54" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="12">
-        <v>2</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="C7" s="14"/>
-      <c r="D7" s="15"/>
-      <c r="E7" s="16"/>
-      <c r="F7" s="17"/>
-    </row>
-    <row r="8" spans="1:6" ht="54" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="12">
-        <v>3</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="C8" s="14"/>
-      <c r="D8" s="15"/>
-      <c r="E8" s="16"/>
-      <c r="F8" s="17"/>
-    </row>
-    <row r="9" spans="1:6" ht="54" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="12">
-        <v>4</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="C9" s="14"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="16"/>
-      <c r="F9" s="17"/>
-    </row>
-    <row r="10" spans="1:6" ht="54" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="12">
-        <v>5</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="C10" s="14"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="16"/>
-      <c r="F10" s="17"/>
-    </row>
-    <row r="12" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
-    </row>
-  </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A12:F12"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -1248,129 +1142,133 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
+      <c r="A1" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
     </row>
     <row r="2" spans="1:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
+      <c r="A2" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
     </row>
     <row r="5" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="G5" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B5" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="D5" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="E5" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="F5" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="G5" s="11" t="s">
-        <v>61</v>
-      </c>
     </row>
     <row r="6" spans="1:7" ht="54" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="12">
+      <c r="A6" s="8">
         <v>1</v>
       </c>
-      <c r="B6" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="C6" s="12">
-        <f>Baseline!D6</f>
-        <v>0</v>
-      </c>
-      <c r="D6" s="15"/>
-      <c r="E6" s="15"/>
-      <c r="F6" s="16"/>
-      <c r="G6" s="17"/>
+      <c r="B6" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="C6" s="8">
+        <v>1</v>
+      </c>
+      <c r="D6" s="10">
+        <v>2</v>
+      </c>
+      <c r="E6" s="10"/>
+      <c r="F6" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="G6" s="15" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="7" spans="1:7" ht="54" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="12">
+      <c r="A7" s="8">
         <v>2</v>
       </c>
-      <c r="B7" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="C7" s="12">
-        <f>Baseline!D7</f>
-        <v>0</v>
-      </c>
-      <c r="D7" s="15"/>
-      <c r="E7" s="15"/>
-      <c r="F7" s="16"/>
-      <c r="G7" s="17"/>
+      <c r="B7" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="C7" s="8">
+        <v>1</v>
+      </c>
+      <c r="D7" s="10">
+        <v>2</v>
+      </c>
+      <c r="E7" s="10"/>
+      <c r="F7" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="G7" s="15" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="8" spans="1:7" ht="54" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="12">
+      <c r="A8" s="8">
         <v>3</v>
       </c>
-      <c r="B8" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="C8" s="12">
-        <f>Baseline!D8</f>
-        <v>0</v>
-      </c>
-      <c r="D8" s="15"/>
-      <c r="E8" s="15"/>
-      <c r="F8" s="16"/>
-      <c r="G8" s="17"/>
+      <c r="B8" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="C8" s="8">
+        <v>1</v>
+      </c>
+      <c r="D8" s="10">
+        <v>2</v>
+      </c>
+      <c r="E8" s="10"/>
+      <c r="F8" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="G8" s="15" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="9" spans="1:7" ht="54" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="12">
+      <c r="A9" s="8">
         <v>4</v>
       </c>
-      <c r="B9" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="C9" s="12">
-        <f>Baseline!D9</f>
-        <v>0</v>
-      </c>
-      <c r="D9" s="15"/>
-      <c r="E9" s="15"/>
-      <c r="F9" s="16"/>
-      <c r="G9" s="17"/>
-    </row>
-    <row r="10" spans="1:7" ht="54" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="12">
-        <v>5</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="C10" s="12">
-        <f>Baseline!D10</f>
-        <v>0</v>
-      </c>
-      <c r="D10" s="15"/>
-      <c r="E10" s="15"/>
-      <c r="F10" s="16"/>
-      <c r="G10" s="17"/>
+      <c r="B9" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="C9" s="8">
+        <v>2</v>
+      </c>
+      <c r="D9" s="10">
+        <v>2</v>
+      </c>
+      <c r="E9" s="10"/>
+      <c r="F9" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="G9" s="15" t="s">
+        <v>103</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1382,9 +1280,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -1394,174 +1292,174 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+    </row>
+    <row r="2" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+    </row>
+    <row r="4" spans="1:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="75.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="8">
+        <v>1</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>104</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="E5" s="19" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="75.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="11">
+        <v>2</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="75.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="8">
+        <v>3</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C7" s="20" t="s">
+        <v>106</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="75.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="8">
+        <v>4</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-    </row>
-    <row r="2" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
+      <c r="D8" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-    </row>
-    <row r="5" spans="1:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="B5" s="11" t="s">
+      <c r="E8" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="C5" s="11" t="s">
+    </row>
+    <row r="9" spans="1:5" ht="78" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="8">
+        <v>5</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="C9" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="E5" s="11" t="s">
+      <c r="D9" s="5" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" ht="75.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="12">
-        <v>1</v>
-      </c>
-      <c r="B6" s="7" t="s">
+      <c r="E9" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="C6" s="9" t="s">
+    </row>
+    <row r="10" spans="1:5" ht="75.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="8">
+        <v>6</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="C10" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="D10" s="5" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" ht="75.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="18">
-        <v>2</v>
-      </c>
-      <c r="B7" s="19" t="s">
+      <c r="E10" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="C7" s="20" t="s">
+    </row>
+    <row r="11" spans="1:5" ht="75.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="8">
+        <v>7</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D7" s="20" t="s">
+      <c r="C11" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="D11" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="E7" s="20" t="s">
+      <c r="E11" s="5" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="75.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="12">
-        <v>3</v>
-      </c>
-      <c r="B8" s="7" t="s">
+    <row r="12" spans="1:5" ht="75.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="8">
+        <v>8</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C12" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D12" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E12" s="5" t="s">
         <v>79</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="75.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="12">
-        <v>4</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="D9" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="E9" s="9" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="78" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="12">
-        <v>5</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="C10" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="D10" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="E10" s="9" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="75.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="18">
-        <v>6</v>
-      </c>
-      <c r="B11" s="19" t="s">
-        <v>88</v>
-      </c>
-      <c r="C11" s="20" t="s">
-        <v>89</v>
-      </c>
-      <c r="D11" s="20" t="s">
-        <v>90</v>
-      </c>
-      <c r="E11" s="20" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="75.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="12">
-        <v>7</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>93</v>
-      </c>
-      <c r="D12" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="E12" s="9" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="75.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="12">
-        <v>8</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="C13" s="9" t="s">
-        <v>97</v>
-      </c>
-      <c r="D13" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="E13" s="9" t="s">
-        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -1574,9 +1472,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -1585,97 +1483,89 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
+      <c r="A1" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
     </row>
     <row r="2" spans="1:3" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-    </row>
-    <row r="5" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="11" t="s">
-        <v>102</v>
-      </c>
-      <c r="B5" s="11" t="s">
-        <v>103</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="64.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="12">
+      <c r="A2" s="18" t="s">
+        <v>81</v>
+      </c>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+    </row>
+    <row r="4" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="64.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="8">
         <v>1</v>
       </c>
-      <c r="B6" s="7" t="s">
-        <v>104</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>105</v>
+      <c r="B5" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="45.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="8">
+        <v>2</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="45.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="12">
-        <v>2</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="45.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="12">
+      <c r="A7" s="8">
         <v>3</v>
       </c>
-      <c r="B8" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="51.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="12">
+      <c r="B7" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="51.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="8">
         <v>4</v>
       </c>
-      <c r="B9" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="45.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="12">
+      <c r="B8" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="45.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="8">
         <v>5</v>
       </c>
-      <c r="B10" s="7" t="s">
-        <v>112</v>
-      </c>
-      <c r="C10" s="9" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="75.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
+      <c r="B9" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>93</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A12:C12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>